<commit_message>
Update meta data for fixed templates
</commit_message>
<xml_diff>
--- a/data/metadata/template import labels.xlsx
+++ b/data/metadata/template import labels.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\mwmi.govuk.data\data\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F36734-5CAB-4783-82FE-462DB88C3A7C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE000AB-91B7-4685-A679-17BBE927F312}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8196" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="template 202204" sheetId="2" r:id="rId1"/>
-    <sheet name="template 202106" sheetId="1" r:id="rId2"/>
+    <sheet name="template 202211" sheetId="3" r:id="rId1"/>
+    <sheet name="template 202204" sheetId="2" r:id="rId2"/>
+    <sheet name="template 202106" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="117">
   <si>
     <t>Year</t>
   </si>
@@ -424,6 +425,16 @@
   </si>
   <si>
     <t>contracts</t>
+  </si>
+  <si>
+    <t>Non-payroll staff;
+Total Contingent labour;
+Headcount</t>
+  </si>
+  <si>
+    <t>Non-payroll staff;
+Total Contingent labour;
+Full-time equivalent</t>
   </si>
 </sst>
 </file>
@@ -1266,6 +1277,777 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{976DBE3B-1844-4070-BC7C-9B95442AFA56}">
+  <dimension ref="A1:E42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="26.77734375" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <f>B7</f>
+        <v>payroll</v>
+      </c>
+      <c r="C8" t="str">
+        <f>C7</f>
+        <v>aao</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" ref="B9:C24" si="0">B8</f>
+        <v>payroll</v>
+      </c>
+      <c r="C9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="0"/>
+        <v>eo</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="0"/>
+        <v>sheo</v>
+      </c>
+      <c r="D12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="0"/>
+        <v>g67</v>
+      </c>
+      <c r="D14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="0"/>
+        <v>scs</v>
+      </c>
+      <c r="D16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="0"/>
+        <v>other</v>
+      </c>
+      <c r="D18" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>payroll</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="0"/>
+        <v>total</v>
+      </c>
+      <c r="D20" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <f t="shared" si="0"/>
+        <v>non payroll</v>
+      </c>
+      <c r="C22" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <f t="shared" si="0"/>
+        <v>non payroll</v>
+      </c>
+      <c r="C23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>non payroll</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="0"/>
+        <v>managers</v>
+      </c>
+      <c r="D24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <f t="shared" ref="B25:C38" si="1">B24</f>
+        <v>non payroll</v>
+      </c>
+      <c r="C25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="1"/>
+        <v>non payroll</v>
+      </c>
+      <c r="C26" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" t="s">
+        <v>41</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="1"/>
+        <v>non payroll</v>
+      </c>
+      <c r="C27" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <f t="shared" si="1"/>
+        <v>non payroll</v>
+      </c>
+      <c r="C28" t="str">
+        <f>C27</f>
+        <v>total</v>
+      </c>
+      <c r="D28" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <f t="shared" si="1"/>
+        <v>non payroll</v>
+      </c>
+      <c r="C29" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" t="s">
+        <v>114</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" t="str">
+        <f>C28</f>
+        <v>total</v>
+      </c>
+      <c r="D30" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <f t="shared" si="1"/>
+        <v>all employees</v>
+      </c>
+      <c r="C31" t="str">
+        <f t="shared" si="1"/>
+        <v>total</v>
+      </c>
+      <c r="D31" t="s">
+        <v>41</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" t="s">
+        <v>61</v>
+      </c>
+      <c r="D32" t="s">
+        <v>53</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <f t="shared" si="1"/>
+        <v>payroll costs</v>
+      </c>
+      <c r="C33" t="s">
+        <v>62</v>
+      </c>
+      <c r="D33" t="s">
+        <v>53</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <f t="shared" si="1"/>
+        <v>payroll costs</v>
+      </c>
+      <c r="C34" t="s">
+        <v>63</v>
+      </c>
+      <c r="D34" t="s">
+        <v>53</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <f t="shared" si="1"/>
+        <v>payroll costs</v>
+      </c>
+      <c r="C35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D35" t="s">
+        <v>53</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <f t="shared" si="1"/>
+        <v>payroll costs</v>
+      </c>
+      <c r="C36" t="s">
+        <v>65</v>
+      </c>
+      <c r="D36" t="s">
+        <v>53</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <f t="shared" si="1"/>
+        <v>payroll costs</v>
+      </c>
+      <c r="C37" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37" t="s">
+        <v>53</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <f t="shared" si="1"/>
+        <v>payroll costs</v>
+      </c>
+      <c r="C38" t="s">
+        <v>57</v>
+      </c>
+      <c r="D38" t="s">
+        <v>53</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>59</v>
+      </c>
+      <c r="C39" t="s">
+        <v>67</v>
+      </c>
+      <c r="D39" t="s">
+        <v>53</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <f t="shared" ref="B40:B41" si="2">B39</f>
+        <v>non payroll costs</v>
+      </c>
+      <c r="C40" t="s">
+        <v>68</v>
+      </c>
+      <c r="D40" t="s">
+        <v>53</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <f t="shared" si="2"/>
+        <v>non payroll costs</v>
+      </c>
+      <c r="C41" t="s">
+        <v>57</v>
+      </c>
+      <c r="D41" t="s">
+        <v>53</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>60</v>
+      </c>
+      <c r="C42" t="str">
+        <f t="shared" ref="C42" si="3">C41</f>
+        <v>total</v>
+      </c>
+      <c r="D42" t="s">
+        <v>53</v>
+      </c>
+      <c r="E42" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE792BE3-088C-488C-8BBC-C131AFCA16F8}">
   <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2036,7 +2818,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>